<commit_message>
feat(database): Add admission form schema and update datatype reference
- Add SQL schema for admission_form table with student records
- Include fields for student identification, course selection, date of birth, and fees
- Update datetype.xlsx with latest reference documentation
- Create database initialization script for admissiondb
</commit_message>
<xml_diff>
--- a/datetype.xlsx
+++ b/datetype.xlsx
@@ -5,16 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sanjana Chaudhary\OneDrive\Documents\sanjanaSQL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\sanjana_SQL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B271A75-3042-4D97-8AF8-88009253C1C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5761C622-45E3-4BBB-842E-0DD6BFB84AE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{477C1697-BC4C-4FA8-8D31-793B09B95072}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{477C1697-BC4C-4FA8-8D31-793B09B95072}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="keys" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="98">
   <si>
     <t>admission fom</t>
   </si>
@@ -295,6 +295,45 @@
   </si>
   <si>
     <t>Joining date</t>
+  </si>
+  <si>
+    <t>keys</t>
+  </si>
+  <si>
+    <t>primay key</t>
+  </si>
+  <si>
+    <t>unique</t>
+  </si>
+  <si>
+    <t>check key</t>
+  </si>
+  <si>
+    <t>foreign key</t>
+  </si>
+  <si>
+    <t>composite key</t>
+  </si>
+  <si>
+    <t>unique value</t>
+  </si>
+  <si>
+    <t>not accept null values</t>
+  </si>
+  <si>
+    <t>accept null vaues</t>
+  </si>
+  <si>
+    <t xml:space="preserve">this is faster then uniques </t>
+  </si>
+  <si>
+    <t>can take only 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can take multipla </t>
+  </si>
+  <si>
+    <t>primary key</t>
   </si>
 </sst>
 </file>
@@ -318,7 +357,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -326,13 +365,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -667,64 +722,64 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{511B8899-7059-472E-AE5E-6B8F7C1780EA}">
-  <dimension ref="A1:O40"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:O44"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.44140625" customWidth="1"/>
-    <col min="2" max="2" width="16.88671875" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" customWidth="1"/>
-    <col min="4" max="4" width="11.33203125" customWidth="1"/>
-    <col min="5" max="5" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.109375" customWidth="1"/>
-    <col min="7" max="7" width="13.77734375" customWidth="1"/>
-    <col min="8" max="8" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.6640625" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" customWidth="1"/>
+    <col min="1" max="1" width="19.42578125" customWidth="1"/>
+    <col min="2" max="2" width="33.140625" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="11.28515625" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" customWidth="1"/>
+    <col min="8" max="8" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" customWidth="1"/>
     <col min="14" max="14" width="25" customWidth="1"/>
-    <col min="15" max="15" width="27.33203125" customWidth="1"/>
+    <col min="15" max="15" width="27.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -768,7 +823,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -794,473 +849,478 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>20</v>
       </c>
-      <c r="N7" t="s">
+      <c r="N11" t="s">
         <v>27</v>
       </c>
-      <c r="O7">
+      <c r="O11">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="N8" t="s">
+      <c r="N12" t="s">
         <v>28</v>
       </c>
-      <c r="O8" t="s">
+      <c r="O12" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>33</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B13" t="s">
         <v>34</v>
       </c>
-      <c r="N9" t="s">
+      <c r="N13" t="s">
         <v>27</v>
       </c>
-      <c r="O9">
+      <c r="O13">
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>36</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B18" t="s">
         <v>42</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C18" t="s">
         <v>43</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D18" t="s">
         <v>44</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E18" t="s">
         <v>45</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F18" t="s">
         <v>46</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G18" t="s">
         <v>47</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H18" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" t="s">
-        <v>39</v>
-      </c>
-      <c r="D15" t="s">
-        <v>49</v>
-      </c>
-      <c r="E15" t="s">
-        <v>49</v>
-      </c>
-      <c r="F15" t="s">
-        <v>39</v>
-      </c>
-      <c r="G15" t="s">
-        <v>38</v>
-      </c>
-      <c r="H15" t="s">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" t="s">
+        <v>49</v>
+      </c>
+      <c r="E19" t="s">
+        <v>49</v>
+      </c>
+      <c r="F19" t="s">
+        <v>39</v>
+      </c>
+      <c r="G19" t="s">
+        <v>38</v>
+      </c>
+      <c r="H19" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B16" t="s">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>37</v>
+      </c>
+      <c r="B20" t="s">
         <v>40</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C20" t="s">
         <v>33</v>
       </c>
-      <c r="D16" t="s">
-        <v>49</v>
-      </c>
-      <c r="E16" t="s">
-        <v>49</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="D20" t="s">
+        <v>49</v>
+      </c>
+      <c r="E20" t="s">
+        <v>49</v>
+      </c>
+      <c r="F20" t="s">
         <v>48</v>
       </c>
-      <c r="G16" t="s">
-        <v>37</v>
-      </c>
-      <c r="H16" t="s">
+      <c r="G20" t="s">
+        <v>37</v>
+      </c>
+      <c r="H20" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>53</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B24" t="s">
         <v>54</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C24" t="s">
         <v>55</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D24" t="s">
         <v>56</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E24" t="s">
         <v>57</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F24" t="s">
         <v>58</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G24" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>38</v>
-      </c>
-      <c r="B21" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" t="s">
-        <v>38</v>
-      </c>
-      <c r="D21" t="s">
-        <v>38</v>
-      </c>
-      <c r="E21" t="s">
-        <v>49</v>
-      </c>
-      <c r="F21" t="s">
-        <v>49</v>
-      </c>
-      <c r="G21" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>37</v>
-      </c>
-      <c r="B22" t="s">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" t="s">
+        <v>39</v>
+      </c>
+      <c r="C25" t="s">
+        <v>38</v>
+      </c>
+      <c r="D25" t="s">
+        <v>38</v>
+      </c>
+      <c r="E25" t="s">
+        <v>49</v>
+      </c>
+      <c r="F25" t="s">
+        <v>49</v>
+      </c>
+      <c r="G25" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" t="s">
         <v>64</v>
       </c>
-      <c r="C22" t="s">
-        <v>37</v>
-      </c>
-      <c r="E22" t="s">
-        <v>49</v>
-      </c>
-      <c r="F22" t="s">
-        <v>49</v>
-      </c>
-      <c r="G22" t="s">
+      <c r="C26" t="s">
+        <v>37</v>
+      </c>
+      <c r="E26" t="s">
+        <v>49</v>
+      </c>
+      <c r="F26" t="s">
+        <v>49</v>
+      </c>
+      <c r="G26" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>61</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B30" t="s">
         <v>54</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C30" t="s">
         <v>62</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D30" t="s">
         <v>56</v>
       </c>
-      <c r="E26" t="s">
-        <v>49</v>
-      </c>
-      <c r="F26" t="s">
+      <c r="E30" t="s">
+        <v>49</v>
+      </c>
+      <c r="F30" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>38</v>
-      </c>
-      <c r="B27" t="s">
-        <v>39</v>
-      </c>
-      <c r="C27" t="s">
-        <v>39</v>
-      </c>
-      <c r="D27" t="s">
-        <v>38</v>
-      </c>
-      <c r="E27" t="s">
-        <v>49</v>
-      </c>
-      <c r="F27" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>37</v>
-      </c>
-      <c r="B28" t="s">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" t="s">
+        <v>39</v>
+      </c>
+      <c r="C31" t="s">
+        <v>39</v>
+      </c>
+      <c r="D31" t="s">
+        <v>38</v>
+      </c>
+      <c r="E31" t="s">
+        <v>49</v>
+      </c>
+      <c r="F31" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C32" t="s">
         <v>65</v>
       </c>
-      <c r="D28" t="s">
-        <v>37</v>
-      </c>
-      <c r="E28" t="s">
+      <c r="D32" t="s">
+        <v>37</v>
+      </c>
+      <c r="E32" t="s">
         <v>13</v>
       </c>
-      <c r="F28" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
+      <c r="F32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>67</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B36" t="s">
         <v>68</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C36" t="s">
         <v>69</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D36" t="s">
         <v>70</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E36" t="s">
         <v>71</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F36" t="s">
         <v>72</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G36" t="s">
         <v>73</v>
       </c>
-      <c r="H32" t="s">
+      <c r="H36" t="s">
         <v>74</v>
       </c>
-      <c r="I32" t="s">
+      <c r="I36" t="s">
         <v>75</v>
       </c>
-      <c r="J32" t="s">
+      <c r="J36" t="s">
         <v>76</v>
       </c>
-      <c r="K32" t="s">
+      <c r="K36" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>38</v>
-      </c>
-      <c r="B33" t="s">
-        <v>39</v>
-      </c>
-      <c r="C33" t="s">
-        <v>38</v>
-      </c>
-      <c r="D33" t="s">
-        <v>39</v>
-      </c>
-      <c r="E33" t="s">
-        <v>38</v>
-      </c>
-      <c r="F33" t="s">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37" t="s">
+        <v>39</v>
+      </c>
+      <c r="C37" t="s">
+        <v>38</v>
+      </c>
+      <c r="D37" t="s">
+        <v>39</v>
+      </c>
+      <c r="E37" t="s">
+        <v>38</v>
+      </c>
+      <c r="F37" t="s">
         <v>51</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G37" t="s">
         <v>51</v>
       </c>
-      <c r="H33" t="s">
+      <c r="H37" t="s">
         <v>51</v>
       </c>
-      <c r="I33" t="s">
-        <v>38</v>
-      </c>
-      <c r="J33" t="s">
-        <v>38</v>
-      </c>
-      <c r="K33" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B34" t="s">
+      <c r="I37" t="s">
+        <v>38</v>
+      </c>
+      <c r="J37" t="s">
+        <v>38</v>
+      </c>
+      <c r="K37" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
         <v>64</v>
       </c>
-      <c r="C34" t="s">
-        <v>37</v>
-      </c>
-      <c r="D34" t="s">
+      <c r="C38" t="s">
+        <v>37</v>
+      </c>
+      <c r="D38" t="s">
         <v>65</v>
       </c>
-      <c r="E34" t="s">
-        <v>37</v>
-      </c>
-      <c r="F34" t="s">
+      <c r="E38" t="s">
+        <v>37</v>
+      </c>
+      <c r="F38" t="s">
         <v>40</v>
       </c>
-      <c r="G34" t="s">
+      <c r="G38" t="s">
         <v>40</v>
       </c>
-      <c r="H34" t="s">
+      <c r="H38" t="s">
         <v>64</v>
       </c>
-      <c r="I34" t="s">
-        <v>37</v>
-      </c>
-      <c r="J34" t="s">
-        <v>37</v>
-      </c>
-      <c r="K34" t="s">
+      <c r="I38" t="s">
+        <v>37</v>
+      </c>
+      <c r="J38" t="s">
+        <v>37</v>
+      </c>
+      <c r="K38" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>79</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B42" t="s">
         <v>80</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C42" t="s">
         <v>35</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D42" t="s">
         <v>81</v>
       </c>
-      <c r="E38" t="s">
+      <c r="E42" t="s">
         <v>84</v>
       </c>
-      <c r="F38" t="s">
+      <c r="F42" t="s">
         <v>82</v>
       </c>
-      <c r="G38" t="s">
+      <c r="G42" t="s">
         <v>83</v>
       </c>
-      <c r="H38" t="s">
+      <c r="H42" t="s">
         <v>73</v>
       </c>
-      <c r="I38" t="s">
+      <c r="I42" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>38</v>
-      </c>
-      <c r="B39" t="s">
-        <v>39</v>
-      </c>
-      <c r="C39" t="s">
-        <v>39</v>
-      </c>
-      <c r="D39" t="s">
-        <v>39</v>
-      </c>
-      <c r="E39" t="s">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>38</v>
+      </c>
+      <c r="B43" t="s">
+        <v>39</v>
+      </c>
+      <c r="C43" t="s">
+        <v>39</v>
+      </c>
+      <c r="D43" t="s">
+        <v>39</v>
+      </c>
+      <c r="E43" t="s">
         <v>13</v>
       </c>
-      <c r="F39" t="s">
-        <v>39</v>
-      </c>
-      <c r="G39" t="s">
-        <v>38</v>
-      </c>
-      <c r="H39" t="s">
+      <c r="F43" t="s">
+        <v>39</v>
+      </c>
+      <c r="G43" t="s">
+        <v>38</v>
+      </c>
+      <c r="H43" t="s">
         <v>51</v>
       </c>
-      <c r="I39" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>37</v>
-      </c>
-      <c r="B40" t="s">
+      <c r="I43" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>37</v>
+      </c>
+      <c r="B44" t="s">
         <v>64</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C44" t="s">
         <v>33</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D44" t="s">
         <v>33</v>
       </c>
-      <c r="E40" t="s">
+      <c r="E44" t="s">
         <v>13</v>
       </c>
-      <c r="F40" t="s">
+      <c r="F44" t="s">
         <v>33</v>
       </c>
-      <c r="G40" t="s">
-        <v>37</v>
-      </c>
-      <c r="H40" t="s">
+      <c r="G44" t="s">
+        <v>37</v>
+      </c>
+      <c r="H44" t="s">
         <v>48</v>
       </c>
-      <c r="I40" t="s">
+      <c r="I44" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1271,15 +1331,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{108D6ACB-DFAE-4805-8B89-740712125C11}">
-  <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J41"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>36</v>
       </c>
@@ -1305,7 +1372,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -1331,7 +1398,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -1357,12 +1424,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>53</v>
       </c>
@@ -1385,7 +1452,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>38</v>
       </c>
@@ -1408,7 +1475,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -1428,12 +1495,12 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>61</v>
       </c>
@@ -1453,7 +1520,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>38</v>
       </c>
@@ -1473,7 +1540,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>37</v>
       </c>
@@ -1493,12 +1560,12 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>67</v>
       </c>
@@ -1530,7 +1597,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>38</v>
       </c>
@@ -1562,7 +1629,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>37</v>
       </c>
@@ -1594,12 +1661,12 @@
         <v>37</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>79</v>
       </c>
@@ -1628,7 +1695,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>38</v>
       </c>
@@ -1657,7 +1724,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>37</v>
       </c>
@@ -1684,6 +1751,60 @@
       </c>
       <c r="I28" t="s">
         <v>65</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>85</v>
+      </c>
+      <c r="B36" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>86</v>
+      </c>
+      <c r="B37" t="s">
+        <v>91</v>
+      </c>
+      <c r="C37" t="s">
+        <v>92</v>
+      </c>
+      <c r="D37" t="s">
+        <v>94</v>
+      </c>
+      <c r="E37" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>87</v>
+      </c>
+      <c r="B38" t="s">
+        <v>91</v>
+      </c>
+      <c r="C38" t="s">
+        <v>93</v>
+      </c>
+      <c r="E38" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>